<commit_message>
refactor: merge payment and direct transaction imports into single template
Direct transactions are now handled by the payments import — if
invoice_document_ref is blank, the system auto-creates invoice + item +
payment. Removes separate direct-transactions-template.xlsx and import
button from calendar page.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/website/public/templates/payments-template.xlsx
+++ b/website/public/templates/payments-template.xlsx
@@ -397,19 +397,21 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K4"/>
+  <dimension ref="A1:M4"/>
   <cols>
-    <col min="1" max="1" width="29.83203125" customWidth="1"/>
+    <col min="1" max="1" width="40.83203125" customWidth="1"/>
     <col min="2" max="2" width="21.83203125" customWidth="1"/>
-    <col min="3" max="3" width="32.83203125" customWidth="1"/>
+    <col min="3" max="3" width="18.83203125" customWidth="1"/>
     <col min="4" max="4" width="14.83203125" customWidth="1"/>
     <col min="5" max="5" width="16.83203125" customWidth="1"/>
     <col min="6" max="6" width="15.83203125" customWidth="1"/>
-    <col min="7" max="7" width="29.83203125" customWidth="1"/>
-    <col min="8" max="8" width="33.83203125" customWidth="1"/>
-    <col min="9" max="9" width="18.83203125" customWidth="1"/>
-    <col min="10" max="10" width="27.83203125" customWidth="1"/>
-    <col min="11" max="11" width="12.83203125" customWidth="1"/>
+    <col min="7" max="7" width="31.83203125" customWidth="1"/>
+    <col min="8" max="8" width="40.83203125" customWidth="1"/>
+    <col min="9" max="9" width="40.83203125" customWidth="1"/>
+    <col min="10" max="10" width="32.83203125" customWidth="1"/>
+    <col min="11" max="11" width="40.83203125" customWidth="1"/>
+    <col min="12" max="12" width="27.83203125" customWidth="1"/>
+    <col min="13" max="13" width="12.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -420,7 +422,7 @@
         <v>direction</v>
       </c>
       <c r="C1" t="str">
-        <v>payment_type</v>
+        <v>partner_name</v>
       </c>
       <c r="D1" t="str">
         <v>payment_date</v>
@@ -435,27 +437,33 @@
         <v>exchange_rate</v>
       </c>
       <c r="H1" t="str">
+        <v>payment_type</v>
+      </c>
+      <c r="I1" t="str">
         <v>bank_account</v>
       </c>
-      <c r="I1" t="str">
-        <v>partner_name</v>
-      </c>
       <c r="J1" t="str">
+        <v>project_code</v>
+      </c>
+      <c r="K1" t="str">
+        <v>category</v>
+      </c>
+      <c r="L1" t="str">
         <v>document_ref</v>
       </c>
-      <c r="K1" t="str">
+      <c r="M1" t="str">
         <v>notes</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Invoice document_ref to pay</v>
+        <v>Invoice document_ref (blank = direct transaction)</v>
       </c>
       <c r="B2" t="str">
         <v>Cash flow direction</v>
       </c>
       <c r="C2" t="str">
-        <v>Payment type</v>
+        <v>Partner name</v>
       </c>
       <c r="D2" t="str">
         <v>Payment date</v>
@@ -470,15 +478,21 @@
         <v>Exchange rate (PEN per USD)</v>
       </c>
       <c r="H2" t="str">
+        <v>Payment type</v>
+      </c>
+      <c r="I2" t="str">
         <v>Bank account (BankName-Last4)</v>
       </c>
-      <c r="I2" t="str">
-        <v>Partner name</v>
-      </c>
       <c r="J2" t="str">
+        <v>Project code (direct txn only)</v>
+      </c>
+      <c r="K2" t="str">
+        <v>Cost category (direct txn only)</v>
+      </c>
+      <c r="L2" t="str">
         <v>Payment receipt reference</v>
       </c>
-      <c r="K2" t="str">
+      <c r="M2" t="str">
         <v>Notes</v>
       </c>
     </row>
@@ -490,7 +504,7 @@
         <v>outbound</v>
       </c>
       <c r="C3" t="str">
-        <v>regular</v>
+        <v>Korakuen SAC</v>
       </c>
       <c r="D3" t="str">
         <v>2026-03-20</v>
@@ -505,27 +519,33 @@
         <v>3.72</v>
       </c>
       <c r="H3" t="str">
+        <v>regular</v>
+      </c>
+      <c r="I3" t="str">
         <v>BCP-1234</v>
       </c>
-      <c r="I3" t="str">
-        <v>Korakuen SAC</v>
-      </c>
       <c r="J3" t="str">
+        <v>PRY001</v>
+      </c>
+      <c r="K3" t="str">
+        <v>materials</v>
+      </c>
+      <c r="L3" t="str">
         <v>PRY001-PY-001</v>
       </c>
-      <c r="K3" t="str">
+      <c r="M3" t="str">
         <v/>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Must exist in DB</v>
+        <v>Must exist in DB if provided</v>
       </c>
       <c r="B4" t="str">
         <v>inbound, outbound</v>
       </c>
       <c r="C4" t="str">
-        <v>regular, detraccion, retencion</v>
+        <v>Must exist in DB</v>
       </c>
       <c r="D4" t="str">
         <v>YYYY-MM-DD</v>
@@ -537,24 +557,30 @@
         <v>USD, PEN</v>
       </c>
       <c r="G4" t="str">
-        <v>Required, 2.5–6.0</v>
+        <v>Auto-filled if blank, 2.5–6.0</v>
       </c>
       <c r="H4" t="str">
-        <v>Required for regular/detraccion</v>
+        <v>regular, detraccion, retencion (default: regular)</v>
       </c>
       <c r="I4" t="str">
-        <v>Must exist in DB</v>
+        <v>Required for regular/detraccion with invoice_document_ref</v>
       </c>
       <c r="J4" t="str">
+        <v>Optional, must exist in DB</v>
+      </c>
+      <c r="K4" t="str">
+        <v>Required for outbound direct transactions</v>
+      </c>
+      <c r="L4" t="str">
         <v>Optional</v>
       </c>
-      <c r="K4" t="str">
+      <c r="M4" t="str">
         <v>Optional</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M4"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: add operation_number to payments (numero de operacion)
Every bank transaction in Peru has an operation number. Added as NOT NULL
for regular/detraccion payments, nullable for retencion (no bank movement).
Wired through schema, migration, views, types, actions, import, and all UI forms.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/website/public/templates/payments-template.xlsx
+++ b/website/public/templates/payments-template.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D29"/>
+  <dimension ref="A1:D30"/>
   <cols>
     <col min="1" max="1" width="28.83203125" customWidth="1"/>
     <col min="2" max="2" width="44.83203125" customWidth="1"/>
@@ -578,27 +578,27 @@
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>bank_account</v>
+        <v>operation_number</v>
       </c>
       <c r="B18" t="str">
-        <v>Yes, for invoice regular/detraccion payments</v>
+        <v>Yes, except retencion</v>
       </c>
       <c r="C18" t="str">
-        <v>Bank account in BankName-Last4 format. Currency must match payment</v>
+        <v>Bank operation/transaction number (numero de operacion)</v>
       </c>
       <c r="D18" t="str">
-        <v>Must exist in DB</v>
+        <v>Free text</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>project_code</v>
+        <v>bank_account</v>
       </c>
       <c r="B19" t="str">
-        <v>No (direct transactions only)</v>
+        <v>Yes, for invoice regular/detraccion payments</v>
       </c>
       <c r="C19" t="str">
-        <v>Project code for direct transactions</v>
+        <v>Bank account in BankName-Last4 format. Currency must match payment</v>
       </c>
       <c r="D19" t="str">
         <v>Must exist in DB</v>
@@ -606,86 +606,100 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>category</v>
+        <v>project_code</v>
       </c>
       <c r="B20" t="str">
-        <v>Yes, for outbound direct transactions</v>
+        <v>No (direct transactions only)</v>
       </c>
       <c r="C20" t="str">
-        <v>Cost category for direct transactions</v>
+        <v>Project code for direct transactions</v>
       </c>
       <c r="D20" t="str">
-        <v>Must match cost_type (project_cost if project_code given, sga otherwise)</v>
+        <v>Must exist in DB</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>document_ref</v>
+        <v>category</v>
       </c>
       <c r="B21" t="str">
-        <v>No</v>
+        <v>Yes, for outbound direct transactions</v>
       </c>
       <c r="C21" t="str">
-        <v>Payment receipt reference</v>
+        <v>Cost category for direct transactions</v>
       </c>
       <c r="D21" t="str">
-        <v/>
+        <v>Must match cost_type (project_cost if project_code given, sga otherwise)</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>notes</v>
+        <v>document_ref</v>
       </c>
       <c r="B22" t="str">
         <v>No</v>
       </c>
       <c r="C22" t="str">
-        <v>Notes</v>
+        <v>Payment receipt reference</v>
       </c>
       <c r="D22" t="str">
         <v/>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" t="str">
-        <v>Notes:</v>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>notes</v>
+      </c>
+      <c r="B23" t="str">
+        <v>No</v>
+      </c>
+      <c r="C23" t="str">
+        <v>Notes</v>
+      </c>
+      <c r="D23" t="str">
+        <v/>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v xml:space="preserve">  - If invoice_document_ref is provided: links payment to an existing invoice</v>
+        <v>Notes:</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v xml:space="preserve">  - If invoice_document_ref is blank: creates a direct transaction (auto-generates invoice + payment)</v>
+        <v xml:space="preserve">  - If invoice_document_ref is provided: links payment to an existing invoice</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v xml:space="preserve">  - partner_name must match an entity tagged as "partner" in the database</v>
+        <v xml:space="preserve">  - If invoice_document_ref is blank: creates a direct transaction (auto-generates invoice + payment)</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v xml:space="preserve">  - Retención only applies to receivable invoices</v>
+        <v xml:space="preserve">  - partner_name must match an entity tagged as "partner" in the database</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
+        <v xml:space="preserve">  - Retención only applies to receivable invoices</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
         <v xml:space="preserve">  - exchange_rate is auto-filled from the database if left blank</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D29"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D30"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:N4"/>
+  <dimension ref="A1:O4"/>
   <cols>
     <col min="1" max="1" width="40.83203125" customWidth="1"/>
     <col min="2" max="2" width="21.83203125" customWidth="1"/>
@@ -697,10 +711,11 @@
     <col min="8" max="8" width="40.83203125" customWidth="1"/>
     <col min="9" max="9" width="40.83203125" customWidth="1"/>
     <col min="10" max="10" width="40.83203125" customWidth="1"/>
-    <col min="11" max="11" width="38.83203125" customWidth="1"/>
-    <col min="12" max="12" width="40.83203125" customWidth="1"/>
-    <col min="13" max="13" width="27.83203125" customWidth="1"/>
-    <col min="14" max="14" width="12.83203125" customWidth="1"/>
+    <col min="11" max="11" width="40.83203125" customWidth="1"/>
+    <col min="12" max="12" width="38.83203125" customWidth="1"/>
+    <col min="13" max="13" width="40.83203125" customWidth="1"/>
+    <col min="14" max="14" width="27.83203125" customWidth="1"/>
+    <col min="15" max="15" width="12.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -732,18 +747,21 @@
         <v>payment_type</v>
       </c>
       <c r="J1" t="str">
+        <v>operation_number</v>
+      </c>
+      <c r="K1" t="str">
         <v>bank_account</v>
       </c>
-      <c r="K1" t="str">
+      <c r="L1" t="str">
         <v>project_code</v>
       </c>
-      <c r="L1" t="str">
+      <c r="M1" t="str">
         <v>category</v>
       </c>
-      <c r="M1" t="str">
+      <c r="N1" t="str">
         <v>document_ref</v>
       </c>
-      <c r="N1" t="str">
+      <c r="O1" t="str">
         <v>notes</v>
       </c>
     </row>
@@ -776,18 +794,21 @@
         <v>Payment type. Defaults to regular if blank</v>
       </c>
       <c r="J2" t="str">
+        <v>Bank operation/transaction number (numero de operacion)</v>
+      </c>
+      <c r="K2" t="str">
         <v>Bank account in BankName-Last4 format. Currency must match payment</v>
       </c>
-      <c r="K2" t="str">
+      <c r="L2" t="str">
         <v>Project code for direct transactions</v>
       </c>
-      <c r="L2" t="str">
+      <c r="M2" t="str">
         <v>Cost category for direct transactions</v>
       </c>
-      <c r="M2" t="str">
+      <c r="N2" t="str">
         <v>Payment receipt reference</v>
       </c>
-      <c r="N2" t="str">
+      <c r="O2" t="str">
         <v>Notes</v>
       </c>
     </row>
@@ -820,18 +841,21 @@
         <v>regular</v>
       </c>
       <c r="J3" t="str">
+        <v>00123456</v>
+      </c>
+      <c r="K3" t="str">
         <v>BCP-1234</v>
       </c>
-      <c r="K3" t="str">
+      <c r="L3" t="str">
         <v>PRY001</v>
       </c>
-      <c r="L3" t="str">
+      <c r="M3" t="str">
         <v>materials</v>
       </c>
-      <c r="M3" t="str">
+      <c r="N3" t="str">
         <v>PRY001-PY-001</v>
       </c>
-      <c r="N3" t="str">
+      <c r="O3" t="str">
         <v/>
       </c>
     </row>
@@ -864,24 +888,27 @@
         <v>regular, detraccion, retencion</v>
       </c>
       <c r="J4" t="str">
-        <v>Must exist in DB</v>
+        <v>Free text</v>
       </c>
       <c r="K4" t="str">
         <v>Must exist in DB</v>
       </c>
       <c r="L4" t="str">
+        <v>Must exist in DB</v>
+      </c>
+      <c r="M4" t="str">
         <v>Must match cost_type (project_cost if project_code given, sga otherwise)</v>
-      </c>
-      <c r="M4" t="str">
-        <v/>
       </c>
       <c r="N4" t="str">
         <v/>
       </c>
+      <c r="O4" t="str">
+        <v/>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:N4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:O4"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: add entity_document_number column to payments import template
Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/website/public/templates/payments-template.xlsx
+++ b/website/public/templates/payments-template.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D30"/>
+  <dimension ref="A1:D31"/>
   <cols>
     <col min="1" max="1" width="28.83203125" customWidth="1"/>
     <col min="2" max="2" width="44.83203125" customWidth="1"/>
@@ -606,100 +606,114 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>project_code</v>
+        <v>entity_document_number</v>
       </c>
       <c r="B20" t="str">
         <v>No (direct transactions only)</v>
       </c>
       <c r="C20" t="str">
-        <v>Project code for direct transactions</v>
+        <v>Supplier/client RUC/DNI for direct transactions</v>
       </c>
       <c r="D20" t="str">
-        <v>Must exist in DB</v>
+        <v>Must exist in DB if provided</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>category</v>
+        <v>project_code</v>
       </c>
       <c r="B21" t="str">
-        <v>Yes, for outbound direct transactions</v>
+        <v>No (direct transactions only)</v>
       </c>
       <c r="C21" t="str">
-        <v>Cost category for direct transactions</v>
+        <v>Project code for direct transactions</v>
       </c>
       <c r="D21" t="str">
-        <v>Must match cost_type (project_cost if project_code given, sga otherwise)</v>
+        <v>Must exist in DB</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>document_ref</v>
+        <v>category</v>
       </c>
       <c r="B22" t="str">
-        <v>No</v>
+        <v>Yes, for outbound direct transactions</v>
       </c>
       <c r="C22" t="str">
-        <v>Payment receipt reference</v>
+        <v>Cost category for direct transactions</v>
       </c>
       <c r="D22" t="str">
-        <v/>
+        <v>Must match cost_type (project_cost if project_code given, sga otherwise)</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>notes</v>
+        <v>document_ref</v>
       </c>
       <c r="B23" t="str">
         <v>No</v>
       </c>
       <c r="C23" t="str">
-        <v>Notes</v>
+        <v>Payment receipt reference</v>
       </c>
       <c r="D23" t="str">
         <v/>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" t="str">
-        <v>Notes:</v>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>notes</v>
+      </c>
+      <c r="B24" t="str">
+        <v>No</v>
+      </c>
+      <c r="C24" t="str">
+        <v>Notes</v>
+      </c>
+      <c r="D24" t="str">
+        <v/>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v xml:space="preserve">  - If invoice_document_ref is provided: links payment to an existing invoice</v>
+        <v>Notes:</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v xml:space="preserve">  - If invoice_document_ref is blank: creates a direct transaction (auto-generates invoice + payment)</v>
+        <v xml:space="preserve">  - If invoice_document_ref is provided: links payment to an existing invoice</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v xml:space="preserve">  - partner_name must match an entity tagged as "partner" in the database</v>
+        <v xml:space="preserve">  - If invoice_document_ref is blank: creates a direct transaction (auto-generates invoice + payment)</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v xml:space="preserve">  - Retención only applies to receivable invoices</v>
+        <v xml:space="preserve">  - partner_name must match an entity tagged as "partner" in the database</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
+        <v xml:space="preserve">  - Retención only applies to receivable invoices</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="str">
         <v xml:space="preserve">  - exchange_rate is auto-filled from the database if left blank</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D30"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D31"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:O4"/>
+  <dimension ref="A1:P4"/>
   <cols>
     <col min="1" max="1" width="40.83203125" customWidth="1"/>
     <col min="2" max="2" width="21.83203125" customWidth="1"/>
@@ -712,10 +726,11 @@
     <col min="9" max="9" width="40.83203125" customWidth="1"/>
     <col min="10" max="10" width="40.83203125" customWidth="1"/>
     <col min="11" max="11" width="40.83203125" customWidth="1"/>
-    <col min="12" max="12" width="38.83203125" customWidth="1"/>
-    <col min="13" max="13" width="40.83203125" customWidth="1"/>
-    <col min="14" max="14" width="27.83203125" customWidth="1"/>
-    <col min="15" max="15" width="12.83203125" customWidth="1"/>
+    <col min="12" max="12" width="40.83203125" customWidth="1"/>
+    <col min="13" max="13" width="38.83203125" customWidth="1"/>
+    <col min="14" max="14" width="40.83203125" customWidth="1"/>
+    <col min="15" max="15" width="27.83203125" customWidth="1"/>
+    <col min="16" max="16" width="12.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -753,15 +768,18 @@
         <v>bank_account</v>
       </c>
       <c r="L1" t="str">
+        <v>entity_document_number</v>
+      </c>
+      <c r="M1" t="str">
         <v>project_code</v>
       </c>
-      <c r="M1" t="str">
+      <c r="N1" t="str">
         <v>category</v>
       </c>
-      <c r="N1" t="str">
+      <c r="O1" t="str">
         <v>document_ref</v>
       </c>
-      <c r="O1" t="str">
+      <c r="P1" t="str">
         <v>notes</v>
       </c>
     </row>
@@ -800,15 +818,18 @@
         <v>Bank account in BankName-Last4 format. Currency must match payment</v>
       </c>
       <c r="L2" t="str">
+        <v>Supplier/client RUC/DNI for direct transactions</v>
+      </c>
+      <c r="M2" t="str">
         <v>Project code for direct transactions</v>
       </c>
-      <c r="M2" t="str">
+      <c r="N2" t="str">
         <v>Cost category for direct transactions</v>
       </c>
-      <c r="N2" t="str">
+      <c r="O2" t="str">
         <v>Payment receipt reference</v>
       </c>
-      <c r="O2" t="str">
+      <c r="P2" t="str">
         <v>Notes</v>
       </c>
     </row>
@@ -847,15 +868,18 @@
         <v>BCP-1234</v>
       </c>
       <c r="L3" t="str">
+        <v>20123456789</v>
+      </c>
+      <c r="M3" t="str">
         <v>PRY001</v>
       </c>
-      <c r="M3" t="str">
+      <c r="N3" t="str">
         <v>materials</v>
       </c>
-      <c r="N3" t="str">
+      <c r="O3" t="str">
         <v>PRY001-PY-001</v>
       </c>
-      <c r="O3" t="str">
+      <c r="P3" t="str">
         <v/>
       </c>
     </row>
@@ -894,21 +918,24 @@
         <v>Must exist in DB</v>
       </c>
       <c r="L4" t="str">
+        <v>Must exist in DB if provided</v>
+      </c>
+      <c r="M4" t="str">
         <v>Must exist in DB</v>
       </c>
-      <c r="M4" t="str">
+      <c r="N4" t="str">
         <v>Must match cost_type (project_cost if project_code given, sga otherwise)</v>
-      </c>
-      <c r="N4" t="str">
-        <v/>
       </c>
       <c r="O4" t="str">
         <v/>
       </c>
+      <c r="P4" t="str">
+        <v/>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:O4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:P4"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>